<commit_message>
fix(lrp/andon): resolve 7-hour time discrepancy in attendance and enforce strict role separation for repair authorization
</commit_message>
<xml_diff>
--- a/prisma/csv/data_shift.xlsx
+++ b/prisma/csv/data_shift.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\0Magang\Toshin-Backend\prisma\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6D69A58D-2708-4A45-8D13-3B95ADE47451}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F50B747F-8E9F-46E2-90C4-46BFC7E7FCF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{6B349DAF-7B8A-41CB-B778-46344149083D}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="25600" windowHeight="14350" xr2:uid="{6B349DAF-7B8A-41CB-B778-46344149083D}"/>
   </bookViews>
   <sheets>
     <sheet name="data_target - Copy" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="19">
   <si>
     <t>id</t>
   </si>
@@ -74,6 +74,9 @@
   </si>
   <si>
     <t>Shift 3</t>
+  </si>
+  <si>
+    <t>Short</t>
   </si>
 </sst>
 </file>
@@ -563,7 +566,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -579,6 +582,9 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -936,7 +942,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46B46F7C-0C86-46FA-B22D-BDA7696EC18E}">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.81640625" style="1" customWidth="1"/>
@@ -1210,6 +1216,35 @@
         <v>0.1</v>
       </c>
     </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" s="1">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="7">
+        <v>0.3125</v>
+      </c>
+      <c r="E10" s="7">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="F10" s="2">
+        <v>60</v>
+      </c>
+      <c r="G10" s="2">
+        <v>10</v>
+      </c>
+      <c r="H10" s="2">
+        <v>10</v>
+      </c>
+      <c r="I10" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: update fitur poin, attendance (HR), dan sinkronisasi shift- Integrasi poin service dan validation
</commit_message>
<xml_diff>
--- a/prisma/csv/data_shift.xlsx
+++ b/prisma/csv/data_shift.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\0Magang\Toshin-Backend\prisma\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F50B747F-8E9F-46E2-90C4-46BFC7E7FCF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E43FADE-5C70-42C3-81DE-E2DB6F4F7B22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="25600" windowHeight="14350" xr2:uid="{6B349DAF-7B8A-41CB-B778-46344149083D}"/>
+    <workbookView xWindow="0" yWindow="930" windowWidth="25600" windowHeight="14350" xr2:uid="{6B349DAF-7B8A-41CB-B778-46344149083D}"/>
   </bookViews>
   <sheets>
     <sheet name="data_target - Copy" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="16">
   <si>
     <t>id</t>
   </si>
@@ -50,15 +50,6 @@
   </si>
   <si>
     <t>Normal</t>
-  </si>
-  <si>
-    <t>Shift 1 (Normal)</t>
-  </si>
-  <si>
-    <t>Shift 2 (Normal)</t>
-  </si>
-  <si>
-    <t>Shift 3 (Normal)</t>
   </si>
   <si>
     <t>Long Shift</t>
@@ -992,7 +983,7 @@
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" s="3">
         <v>0.3125</v>
@@ -1021,7 +1012,7 @@
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D3" s="3">
         <v>0.64583333333333337</v>
@@ -1050,7 +1041,7 @@
         <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D4" s="3">
         <v>0.97916666666666663</v>
@@ -1076,10 +1067,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D5" s="3">
         <v>0.3125</v>
@@ -1105,10 +1096,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D6" s="3">
         <v>0.8125</v>
@@ -1134,10 +1125,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C7" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D7" s="3">
         <v>0.3125</v>
@@ -1163,10 +1154,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D8" s="3">
         <v>0.64583333333333337</v>
@@ -1192,10 +1183,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D9" s="3">
         <v>0.97916666666666663</v>
@@ -1221,10 +1212,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D10" s="7">
         <v>0.3125</v>

</xml_diff>